<commit_message>
Resolve W03 E01 multicollinearity and update methodology
</commit_message>
<xml_diff>
--- a/methodology/Methodology_Decision_Table.xlsx
+++ b/methodology/Methodology_Decision_Table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a261b646168a133d/Documents/IUS - Data Science/2026 - Fall/SENIOR THESIS/output/methodology/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a261b646168a133d/Documents/GitHub/weathering-the-yield/methodology/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="8_{E2880474-6383-4A23-83FB-0BFB047B2884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2C5CE2F-5450-4276-B032-21B326277615}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{E2880474-6383-4A23-83FB-0BFB047B2884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE039F8-36F8-4ED2-A89A-561356D8C01A}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="382">
   <si>
     <t>Senior Thesis Methodology Decision Table</t>
   </si>
@@ -255,22 +255,7 @@
     <t>What will Model Group 3 add?</t>
   </si>
   <si>
-    <t>A limited set of approximately 3–5 interpretable heat and moisture extreme indicators</t>
-  </si>
-  <si>
-    <t>Sabut et al. (2025); Ting et al. (2023); Li et al. (2019); Kim et al. (2024)</t>
-  </si>
-  <si>
-    <t>Tests whether engineered extremes add information beyond conventional weather.</t>
-  </si>
-  <si>
     <t>Thresholds and definitions cannot be selected from final holdout performance.</t>
-  </si>
-  <si>
-    <t>Extreme-feature script</t>
-  </si>
-  <si>
-    <t>Exact features will be documented in Sheet 2.</t>
   </si>
   <si>
     <t>M09</t>
@@ -905,9 +890,6 @@
     <t>https://doi.org/10.1038/s41598-023-27931-7 ; https://doi.org/10.1016/j.scitotenv.2024.175898</t>
   </si>
   <si>
-    <t>Tree-based models can learn interactions among E01–E04 directly. An explicit interaction could be reserved for a secondary sensitivity analysis if justified using pre-2022 development data.</t>
-  </si>
-  <si>
     <t>Compound heat and moisture stress is biologically plausible, but precipitation does not directly measure soil or crop water status and the four selected extremes already represent the major stress families.</t>
   </si>
   <si>
@@ -1106,9 +1088,6 @@
     <t>https://doi.org/10.1016/j.agrformet.2025.110632 ; https://doi.org/10.1016/j.agrformet.2024.110286 ; https://doi.org/10.1016/j.scitotenv.2024.175898</t>
   </si>
   <si>
-    <t>Represents frequency of high-temperature exposure during the reproductive-sensitive period.</t>
-  </si>
-  <si>
     <t>Sabut et al. (2025); Lingua et al. (2024); Niu et al. (2024)</t>
   </si>
   <si>
@@ -1196,12 +1175,6 @@
     <t>Initial training begins in 2001 after lag-1 yield was selected as the recent-history predictor. The earlier 2003 start was used only for the M06 candidate comparison because the alternative 3-year history feature required three preceding years.</t>
   </si>
   <si>
-    <t>Development-data audit identified a strong correlation with E01 hot-day count (r = 0.95). Both are retained because they represent different concepts; multicollinearity will be evaluated during linear-model development using pre-2022 data.</t>
-  </si>
-  <si>
-    <t>Development-data audit confirmed substantial variation. Strong correlation with W03 July mean temperature (r = 0.95) will be evaluated for multicollinearity during linear-model development; feature retained because it represents threshold-based heat frequency rather than average temperature.</t>
-  </si>
-  <si>
     <t>Development-data audit found nonzero exposure in 287 of 2,024 county-years (14.2%). Although sparse, the feature captures severe heat events and is not redundant with E01 (overall r = 0.41; r = 0.60 among nonzero E02 observations). Retained.</t>
   </si>
   <si>
@@ -1209,6 +1182,37 @@
   </si>
   <si>
     <t>Development-data audit showed adequate variation (24.5–254 mm; median 75.5 mm) and plausible clustered extreme events. Retained without modification.</t>
+  </si>
+  <si>
+    <t>Three retained extreme-weather indicators: E02 reproductive-period extreme heat accumulation, E03 longest July–August dry spell, and E04 maximum May–July rolling 5-day precipitation. E01 hot-day count was evaluated but excluded following development-period multicollinearity and sensitivity analysis.</t>
+  </si>
+  <si>
+    <t>Tests whether engineered extremes add predictive information beyond conventional weather while limiting redundant predictors. E01 was highly correlated with W03 and did not improve rolling-origin predictive performance when retained.</t>
+  </si>
+  <si>
+    <t>Sabut et al. (2025); Ting et al. (2023); Li et al. (2019); Kim et al. (2024); 
+Advisor feedback; development-period W03/E01 multicollinearity and rolling-origin sensitivity analysis</t>
+  </si>
+  <si>
+    <t>E01 remains documented in Sheet 2 and in the engineered-weather dataset for reproducibility but is excluded from the primary modeling predictor set. The exclusion decision was made using pre-2022 development data only; the 2022–2025 final holdout was not used.</t>
+  </si>
+  <si>
+    <t>Weather feature engineering and multicollinearity sensitivity analysis scripts</t>
+  </si>
+  <si>
+    <t>Development-period modeling confirmed strong correlation with E01 hot-day count (r = 0.951; W03 VIF = 17.3). A 2012–2021 rolling-origin sensitivity analysis compared models containing both W03 and E01, W03 without E01, and E01 without W03. The W03-only specification produced the lowest mean RMSE (20.5) and MAE (17.7) and had the lowest RMSE in 8 of 10 validation years and lowest MAE in 9 of 10 years. W03 was retained and E01 was excluded before final holdout evaluation.</t>
+  </si>
+  <si>
+    <t>Initially selected as a literature-supported measure of high-temperature frequency during the reproductive-sensitive period. Development-period analysis showed that E01 was highly redundant with W03 July mean temperature and did not improve rolling-origin predictive performance when both variables were retained.</t>
+  </si>
+  <si>
+    <t>No for feature calculation — fixed literature threshold. The exclusion decision was based only on pre-2022 development data.</t>
+  </si>
+  <si>
+    <t>Strong correlation with W03 was confirmed in the common modeling sample (r = 0.951; E01 VIF = 16.0). In 2012–2021 rolling-origin validation, the W03-only specification had mean RMSE = 20.5 and mean MAE = 17.7, compared with RMSE = 21.1 and MAE = 18.3 when both variables were included and RMSE = 21.4 and MAE = 18.6 when E01 was retained without W03. E01 was excluded before evaluation of the 2022–2025 holdout but remains documented and engineered for reproducibility.</t>
+  </si>
+  <si>
+    <t>Tree-based models can learn interactions among the retained conventional and extreme-weather predictors directly. An explicit interaction term is therefore not included in the primary feature set.</t>
   </si>
 </sst>
 </file>
@@ -1513,10 +1517,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MethodologyDecisionsTable" displayName="MethodologyDecisionsTable" ref="A10:K32" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="11">
@@ -2032,10 +2032,10 @@
         <v>57</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>5</v>
@@ -2044,19 +2044,19 @@
         <v>58</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="J15" s="5">
         <v>46266</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="175.5">
@@ -2067,31 +2067,31 @@
         <v>60</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="J16" s="5">
         <v>46266</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="40.5">
@@ -2127,7 +2127,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="27">
+    <row r="18" spans="1:11" ht="94.5">
       <c r="A18" s="4" t="s">
         <v>70</v>
       </c>
@@ -2138,515 +2138,517 @@
         <v>72</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>73</v>
+        <v>372</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>74</v>
+        <v>374</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>75</v>
+        <v>373</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="J18" s="5"/>
+        <v>376</v>
+      </c>
+      <c r="J18" s="5">
+        <v>46287</v>
+      </c>
       <c r="K18" s="4" t="s">
-        <v>78</v>
+        <v>375</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="40.5">
       <c r="A19" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="162">
       <c r="A20" s="4" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="J20" s="5">
         <v>46279</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="27">
       <c r="A21" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J21" s="5">
         <v>46279</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="40.5">
       <c r="A22" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J22" s="5">
         <v>46279</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="40.5">
       <c r="A23" s="4" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="J23" s="5">
         <v>46279</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="40.5">
       <c r="A24" s="4" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="J24" s="5">
         <v>46279</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="40.5">
       <c r="A25" s="4" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="J25" s="5">
         <v>46279</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="40.5">
       <c r="A26" s="4" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="J26" s="5">
         <v>46279</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="40.5">
       <c r="A27" s="4" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="J27" s="5">
         <v>46279</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="81">
       <c r="A28" s="4" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="J28" s="5"/>
       <c r="K28" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="40.5">
       <c r="A29" s="4" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="J29" s="5"/>
       <c r="K29" s="4" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="54">
       <c r="A30" s="4" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="J30" s="5">
         <v>46279</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="40.5">
       <c r="A31" s="4" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="J31" s="5">
         <v>46279</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="40.5">
       <c r="A32" s="4" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="J32" s="5">
         <v>46279</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="18" customHeight="1">
       <c r="A34" s="20" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B34" s="20"/>
       <c r="C34" s="20"/>
@@ -2712,7 +2714,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="14" customHeight="1">
       <c r="A1" s="12" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -2746,7 +2748,7 @@
     </row>
     <row r="4" spans="1:13" ht="27.75">
       <c r="A4" s="10" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>3</v>
@@ -2770,10 +2772,10 @@
       </c>
       <c r="B5" s="6">
         <f>COUNTIF(I11:I200,"Final")</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
@@ -2806,11 +2808,11 @@
     </row>
     <row r="7" spans="1:13" ht="14" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(I11:I200,"Excluded")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
@@ -2825,34 +2827,34 @@
     </row>
     <row r="10" spans="1:13" ht="16.05" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="I10" s="10" t="s">
         <v>13</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>15</v>
@@ -2861,704 +2863,704 @@
         <v>19</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="81">
       <c r="A11" s="7" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="67.5">
       <c r="A12" s="9" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>226</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>231</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="54">
       <c r="A13" s="7" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="40.5">
       <c r="A14" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="H14" s="7" t="s">
         <v>257</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>372</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>262</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="40.5">
       <c r="A15" s="9" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J15" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="M15" s="9" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="148.5">
+      <c r="A16" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="K15" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="L15" s="9" t="s">
-        <v>367</v>
-      </c>
-      <c r="M15" s="9" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="81">
-      <c r="A16" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>268</v>
-      </c>
       <c r="D16" s="7" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="40.5">
       <c r="A17" s="9" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="40.5">
       <c r="A18" s="7" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="40.5">
       <c r="A19" s="9" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="94.5">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="148.5">
       <c r="A20" s="7" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>5</v>
+        <v>248</v>
       </c>
       <c r="J20" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="M20" s="7" t="s">
         <v>339</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>346</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>377</v>
-      </c>
-      <c r="M20" s="7" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="81">
       <c r="A21" s="9" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="54">
       <c r="A22" s="7" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="54">
       <c r="A23" s="9" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="54">
       <c r="A24" s="7" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="M24" s="7" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="54">
       <c r="A25" s="9" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B25" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>306</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>304</v>
-      </c>
       <c r="I25" s="11" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="54">
       <c r="A26" s="7" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="67.5">
       <c r="A27" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>279</v>
+        <v>381</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update methodology decision table through development-stage lock
Updated the methodology decision table to reflect completed Week 4 modeling decisions.

- Finalized the model-family comparison as Linear Regression, Random Forest, and XGBoost
- Documented Linear Regression with Group 3 predictors as the selected development-stage model
- Added the difficult-year diagnostic methodology for 2012, 2013, and 2015
- Documented the formal pre-holdout development-stage lock
- Updated supporting validation, reproducibility, and leakage-control notes
- Confirmed the 2022-2025 final holdout remains unused
</commit_message>
<xml_diff>
--- a/methodology/Methodology_Decision_Table.xlsx
+++ b/methodology/Methodology_Decision_Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a261b646168a133d/Documents/GitHub/weathering-the-yield/methodology/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{E2880474-6383-4A23-83FB-0BFB047B2884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE039F8-36F8-4ED2-A89A-561356D8C01A}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="8_{E2880474-6383-4A23-83FB-0BFB047B2884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AA9E37-1F37-4E99-A488-36B950B68385}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Methodology Decisions" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="409">
   <si>
     <t>Senior Thesis Methodology Decision Table</t>
   </si>
@@ -297,9 +297,6 @@
     <t>Hewamalage et al. (2023); Stracqualursi (2026); advisor feedback</t>
   </si>
   <si>
-    <t>Model development script</t>
-  </si>
-  <si>
     <t>M11</t>
   </si>
   <si>
@@ -321,12 +318,6 @@
     <t>Must remain unused for feature selection, tuning, or threshold selection.</t>
   </si>
   <si>
-    <t>Final analysis script</t>
-  </si>
-  <si>
-    <t>Evaluate only after methodology and model choices are locked.</t>
-  </si>
-  <si>
     <t>M12</t>
   </si>
   <si>
@@ -366,21 +357,12 @@
     <t>Use the same observed county-years, training periods, validation years, preprocessing rules, algorithms, and metrics for all groups</t>
   </si>
   <si>
-    <t>Advisor feedback; literature review</t>
-  </si>
-  <si>
     <t>Ensures differences reflect predictor information rather than evaluation differences.</t>
   </si>
   <si>
     <t>No model group should receive information unavailable to the others except its intended added predictors.</t>
   </si>
   <si>
-    <t>Model comparison script</t>
-  </si>
-  <si>
-    <t>One of Dr. R's explicit recommendations.</t>
-  </si>
-  <si>
     <t>M14</t>
   </si>
   <si>
@@ -432,9 +414,6 @@
     <t>Evaluation script</t>
   </si>
   <si>
-    <t>Avoid ranking models on R² alone.</t>
-  </si>
-  <si>
     <t>M16</t>
   </si>
   <si>
@@ -525,24 +504,6 @@
     <t>Which modeling algorithms will be considered?</t>
   </si>
   <si>
-    <t>Multiple linear regression plus a limited set of tree-based ML methods such as Random Forest and gradient boosting/XGBoost</t>
-  </si>
-  <si>
-    <t>Project scope; crop prediction literature</t>
-  </si>
-  <si>
-    <t>Provides an interpretable benchmark plus nonlinear alternatives without excessive model proliferation.</t>
-  </si>
-  <si>
-    <t>Hyperparameter tuning must occur within pre-2022 development validation.</t>
-  </si>
-  <si>
-    <t>Modeling scripts</t>
-  </si>
-  <si>
-    <t>Final algorithm set should remain small.</t>
-  </si>
-  <si>
     <t>M20</t>
   </si>
   <si>
@@ -555,21 +516,12 @@
     <t>Feature definitions and tuning decisions may use literature and pre-2022 development results only; final 2022–2025 results cannot drive feature selection</t>
   </si>
   <si>
-    <t>Forecast evaluation literature; advisor guidance</t>
-  </si>
-  <si>
     <t>Protects against test-set overfitting and hindsight-driven methodology.</t>
   </si>
   <si>
     <t>Final holdout cannot be reopened during feature engineering.</t>
   </si>
   <si>
-    <t>Decision log + modeling workflow</t>
-  </si>
-  <si>
-    <t>One of the most important methodological safeguards.</t>
-  </si>
-  <si>
     <t>M21</t>
   </si>
   <si>
@@ -616,12 +568,6 @@
   </si>
   <si>
     <t>Any manual intervention should be documented.</t>
-  </si>
-  <si>
-    <t>Project folders / scripts / decision log</t>
-  </si>
-  <si>
-    <t>Decision Log sheet will be part of this process.</t>
   </si>
   <si>
     <t>Use this sheet as the high-level methodology control document. Finalize provisional decisions only from published literature, pre-2022 development data, or advisor feedback—never from 2022–2025 final holdout performance.</t>
@@ -677,9 +623,6 @@
     <t>How should recent county yield history be represented?</t>
   </si>
   <si>
-    <t>Forward-looking expanding-window rolling-origin validation using only pre-2022 observations. The initial development training window will use 2003–2011 common-sample observations, with 2012 as the first validation year. The training window will then expand one year at a time through the final 2021 development validation fold.</t>
-  </si>
-  <si>
     <t>For each fold, only observations preceding the validation year may be used for model fitting, preprocessing, feature estimation, or tuning. The 2022–2025 final holdout remains untouched during development.</t>
   </si>
   <si>
@@ -1213,6 +1156,144 @@
   </si>
   <si>
     <t>Tree-based models can learn interactions among the retained conventional and extreme-weather predictors directly. An explicit interaction term is therefore not included in the primary feature set.</t>
+  </si>
+  <si>
+    <t>Forward-looking expanding-window rolling-origin validation using only pre-2022 observations. The initial development training window uses 2001–2011 observations, with 2012 as the first validation year. The training window then expands one year at a time through the final 2021 development validation fold.</t>
+  </si>
+  <si>
+    <t>Scripts 17–20 development-stage model evaluation and comparison</t>
+  </si>
+  <si>
+    <t>Final holdout evaluation workflow following development-stage lock</t>
+  </si>
+  <si>
+    <t>Development-stage algorithm, predictor group, exact model formula, and predictor definitions were formally locked in Script 22 before final holdout evaluation. At the completion of Script 22, the 2022–2025 holdout remained unused.</t>
+  </si>
+  <si>
+    <t>Advisor feedback; literature review; Scripts 17–20 development-stage model comparison</t>
+  </si>
+  <si>
+    <t>Scripts 17–20 common expanding-window comparison workflow</t>
+  </si>
+  <si>
+    <t>All nine algorithm × predictor-group specifications were evaluated over the same 2012–2021 validation years. Each pooled specification contained 739 validation observations.</t>
+  </si>
+  <si>
+    <t>Model selection continued to prioritize pooled RMSE, with MAE used as a complementary error measure and R² treated as secondary. The selected Linear Regression Group 3 specification ranked first among all nine development-stage specifications on pooled RMSE, MAE, and R².</t>
+  </si>
+  <si>
+    <t>Multiple Linear Regression, Random Forest, and XGBoost</t>
+  </si>
+  <si>
+    <t>Project scope; crop prediction literature; Scripts 17–20 development-stage model comparison</t>
+  </si>
+  <si>
+    <t>Provides an interpretable linear benchmark plus two nonlinear tree-based ensemble alternatives while keeping the model-family comparison limited and computationally manageable.</t>
+  </si>
+  <si>
+    <t>Hyperparameter tuning must occur entirely within pre-2022 development validation.</t>
+  </si>
+  <si>
+    <t>Scripts 17–20 development-stage model fitting, tuning, and comparison</t>
+  </si>
+  <si>
+    <t>The algorithm set is closed before final holdout evaluation. No additional model families will be introduced based on 2022–2025 performance.</t>
+  </si>
+  <si>
+    <t>Scripts 21–22 difficult-year diagnostic and development-stage lock</t>
+  </si>
+  <si>
+    <t>Decision log + modeling workflow + development-stage lock</t>
+  </si>
+  <si>
+    <t>Script 21 was descriptive and diagnostic only and did not trigger predictor, threshold, or model changes. Script 22 formally locked the predictor set and model specification before final holdout evaluation.</t>
+  </si>
+  <si>
+    <t>Project folders / scripts / methodology decision table / output/development_stage_lock/</t>
+  </si>
+  <si>
+    <t>Script 22 created a machine-readable pre-holdout checkpoint including development_stage_lock.csv, overall_development_ranking.csv, numeric_selection_difference.csv, locked_predictor_definition.csv, development_stage_lock_object.rds, and pre_holdout_checkpoint.csv.</t>
+  </si>
+  <si>
+    <t>M23</t>
+  </si>
+  <si>
+    <t>Model selection</t>
+  </si>
+  <si>
+    <t>Which development-stage model specification will advance to final holdout evaluation?</t>
+  </si>
+  <si>
+    <t>Linear Regression with Group 3 predictors: historical baseline predictors plus W01–W06 conventional weather variables and E02–E04 retained extreme-weather indicators.</t>
+  </si>
+  <si>
+    <t>Scripts 17–20 development-stage model comparison; pooled 2012–2021 expanding-window validation results</t>
+  </si>
+  <si>
+    <t>Linear Regression Group 3 produced the strongest overall development-stage performance. Pooled RMSE was 22.56 bu/acre, pooled MAE was 18.10 bu/acre, and pooled R² was 0.553. It ranked first among all nine algorithm × predictor-group specifications on all three pooled metrics and was the best overall specification in 6 of 10 validation years. In the sensitivity analysis excluding 2012, it remained first with mean RMSE of 19.5 and mean MAE of 16.8.</t>
+  </si>
+  <si>
+    <t>Selection was based exclusively on pre-2022 development results. No 2022–2025 holdout observations were used to select the algorithm or predictor group.</t>
+  </si>
+  <si>
+    <t>Script 20 model-family comparison; Script 22 development-stage lock</t>
+  </si>
+  <si>
+    <t>The final locked specification uses factor(fips), year_centered, lag1_yield, W01–W06, and E02–E04. The specification must not be altered in response to final holdout performance.</t>
+  </si>
+  <si>
+    <t>M24</t>
+  </si>
+  <si>
+    <t>Diagnostic evaluation</t>
+  </si>
+  <si>
+    <t>How will unusually difficult development validation years be identified and interpreted?</t>
+  </si>
+  <si>
+    <t>Identify the three validation years with the highest median RMSE across all nine algorithm × predictor-group specifications, then descriptively examine observed yield behavior, model performance, and weather conditions without using the diagnostic for additional tuning.</t>
+  </si>
+  <si>
+    <t>Advisor feedback; Script 21 difficult-year diagnostic</t>
+  </si>
+  <si>
+    <t>Using median RMSE across the complete modeling framework identifies years that were consistently difficult rather than selecting years visually or because one particular model performed poorly. Median RMSE also limits the influence of one exceptionally poor specification.</t>
+  </si>
+  <si>
+    <t>The diagnostic uses development-period validation results only. It cannot use 2022–2025 data or trigger additional predictor selection, algorithm selection, or tuning.</t>
+  </si>
+  <si>
+    <t>21_difficult_year_diagnostic.R</t>
+  </si>
+  <si>
+    <t>The systematic rule identified 2012, 2013, and 2015. These years exhibited different yield and weather profiles rather than one common difficult-year pattern. No model or predictor changes were made after the diagnostic.</t>
+  </si>
+  <si>
+    <t>M25</t>
+  </si>
+  <si>
+    <t>Development-stage lock</t>
+  </si>
+  <si>
+    <t>When and how will model-development choices be frozen before final evaluation?</t>
+  </si>
+  <si>
+    <t>After development-stage model comparison and the planned difficult-year diagnostic are complete, formally lock the selected algorithm, predictor group, exact model formula, predictor definitions, and development-stage selection evidence before loading or evaluating the 2022–2025 holdout.</t>
+  </si>
+  <si>
+    <t>Scripts 20–22; leakage safeguards established in M11 and M20</t>
+  </si>
+  <si>
+    <t>Creates an auditable boundary between model development and final evaluation and prevents post-holdout changes to the modeling strategy.</t>
+  </si>
+  <si>
+    <t>The 2022–2025 holdout must remain unused until the development-stage lock has been written and verified.</t>
+  </si>
+  <si>
+    <t>22_development_stage_lock.R; output/development_stage_lock/</t>
+  </si>
+  <si>
+    <t>Script 22 locked Linear Regression + Group 3. No new model fitting, tuning, or predictor changes occurred in Script 22, and the checkpoint explicitly records final_holdout_used = FALSE.</t>
   </si>
 </sst>
 </file>
@@ -1517,8 +1598,12 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MethodologyDecisionsTable" displayName="MethodologyDecisionsTable" ref="A10:K32" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MethodologyDecisionsTable" displayName="MethodologyDecisionsTable" ref="A10:K35" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Decision ID" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Category" dataDxfId="15"/>
@@ -1731,7 +1816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="11" style="3" customWidth="1"/>
@@ -1801,8 +1886,8 @@
         <v>5</v>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(E11:E32,"Final")</f>
-        <v>20</v>
+        <f>COUNTIF(E11:E35,"Final")</f>
+        <v>24</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>6</v>
@@ -1820,8 +1905,8 @@
         <v>7</v>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF(E11:E32,"Provisional")</f>
-        <v>2</v>
+        <f>COUNTIF(E11:E35,"Provisional")</f>
+        <v>1</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="19"/>
@@ -1837,7 +1922,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(E11:E32,"Needs Advisor Input")</f>
+        <f>COUNTIF(E11:E35,"Needs Advisor Input")</f>
         <v>0</v>
       </c>
       <c r="D7" s="19"/>
@@ -2032,10 +2117,10 @@
         <v>57</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>5</v>
@@ -2044,19 +2129,19 @@
         <v>58</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="J15" s="5">
         <v>46266</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>366</v>
+        <v>347</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="175.5">
@@ -2067,31 +2152,31 @@
         <v>60</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>205</v>
+        <v>186</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>206</v>
+        <v>187</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>208</v>
+        <v>189</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>209</v>
+        <v>190</v>
       </c>
       <c r="J16" s="5">
         <v>46266</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>210</v>
+        <v>191</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="40.5">
@@ -2138,28 +2223,28 @@
         <v>72</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>372</v>
+        <v>353</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>374</v>
+        <v>355</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>373</v>
+        <v>354</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>73</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>376</v>
+        <v>357</v>
       </c>
       <c r="J18" s="5">
         <v>46287</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>375</v>
+        <v>356</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="40.5">
@@ -2206,7 +2291,7 @@
         <v>85</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>203</v>
+        <v>363</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>5</v>
@@ -2215,451 +2300,558 @@
         <v>86</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>367</v>
+        <v>348</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>204</v>
+        <v>185</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>87</v>
+        <v>364</v>
       </c>
       <c r="J20" s="5">
         <v>46279</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="27">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="94.5">
       <c r="A21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="E21" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F21" s="4" t="s">
+      <c r="G21" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="H21" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="H21" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="I21" s="4" t="s">
-        <v>95</v>
+        <v>365</v>
       </c>
       <c r="J21" s="5">
         <v>46279</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>96</v>
+        <v>366</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="40.5">
       <c r="A22" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="E22" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="G22" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="H22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F22" s="4" t="s">
+      <c r="I22" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="J22" s="5">
         <v>46279</v>
       </c>
       <c r="K22" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="67.5">
+      <c r="A23" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="40.5">
-      <c r="A23" s="4" t="s">
+      <c r="D23" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="E23" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="H23" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>112</v>
-      </c>
       <c r="I23" s="4" t="s">
-        <v>113</v>
+        <v>368</v>
       </c>
       <c r="J23" s="5">
         <v>46279</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>114</v>
+        <v>369</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="40.5">
       <c r="A24" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="I24" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>122</v>
       </c>
       <c r="J24" s="5">
         <v>46279</v>
       </c>
       <c r="K24" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="108">
+      <c r="A25" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="40.5">
-      <c r="A25" s="4" t="s">
+      <c r="H25" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="I25" s="4" t="s">
         <v>125</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="I25" s="4" t="s">
-        <v>131</v>
       </c>
       <c r="J25" s="5">
         <v>46279</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>132</v>
+        <v>370</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="40.5">
       <c r="A26" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="I26" s="4" t="s">
         <v>133</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>140</v>
       </c>
       <c r="J26" s="5">
         <v>46279</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="40.5">
       <c r="A27" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I27" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="I27" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="J27" s="5">
         <v>46279</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="81">
       <c r="A28" s="4" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="J28" s="5"/>
       <c r="K28" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="67.5">
+      <c r="A29" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="J29" s="5">
+        <v>46302</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="81">
+      <c r="A30" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" ht="40.5">
-      <c r="A29" s="4" t="s">
+      <c r="E30" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="G30" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="H30" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="I29" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="J29" s="5"/>
-      <c r="K29" s="4" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="54">
-      <c r="A30" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="H30" s="4" t="s">
-        <v>175</v>
-      </c>
       <c r="I30" s="4" t="s">
-        <v>176</v>
+        <v>378</v>
       </c>
       <c r="J30" s="5">
         <v>46279</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>177</v>
+        <v>379</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="40.5">
       <c r="A31" s="4" t="s">
-        <v>178</v>
+        <v>162</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="J31" s="5">
         <v>46279</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="40.5">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="108">
       <c r="A32" s="4" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>194</v>
+        <v>380</v>
       </c>
       <c r="J32" s="5">
         <v>46279</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="18" customHeight="1">
-      <c r="A34" s="20" t="s">
-        <v>196</v>
-      </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20"/>
-      <c r="J34" s="20"/>
-      <c r="K34" s="20"/>
+        <v>381</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="148.5">
+      <c r="A33" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="J33" s="5">
+        <v>46302</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="94.5">
+      <c r="A34" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="J34" s="5">
+        <v>46302</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="81">
+      <c r="A35" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="J35" s="5">
+        <v>46302</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="18" customHeight="1">
+      <c r="A37" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="20"/>
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2667,9 +2859,9 @@
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="D4:K4"/>
     <mergeCell ref="D5:K7"/>
-    <mergeCell ref="A34:K34"/>
+    <mergeCell ref="A37:K37"/>
   </mergeCells>
-  <conditionalFormatting sqref="E11:E32">
+  <conditionalFormatting sqref="E11:E35">
     <cfRule type="expression" dxfId="5" priority="1">
       <formula>E11="Final"</formula>
     </cfRule>
@@ -2681,7 +2873,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="E11:E32" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="E11:E35" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Final,Provisional,Needs Advisor Input"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2714,7 +2906,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="14" customHeight="1">
       <c r="A1" s="12" t="s">
-        <v>251</v>
+        <v>232</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -2748,7 +2940,7 @@
     </row>
     <row r="4" spans="1:13" ht="27.75">
       <c r="A4" s="10" t="s">
-        <v>250</v>
+        <v>231</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>3</v>
@@ -2775,7 +2967,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>249</v>
+        <v>230</v>
       </c>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
@@ -2808,7 +3000,7 @@
     </row>
     <row r="7" spans="1:13" ht="14" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(I11:I200,"Excluded")</f>
@@ -2827,34 +3019,34 @@
     </row>
     <row r="10" spans="1:13" ht="16.05" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>247</v>
+        <v>228</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>246</v>
+        <v>227</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>245</v>
+        <v>226</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>244</v>
+        <v>225</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>243</v>
+        <v>224</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>242</v>
+        <v>223</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>241</v>
+        <v>222</v>
       </c>
       <c r="I10" s="10" t="s">
         <v>13</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>15</v>
@@ -2863,704 +3055,704 @@
         <v>19</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>239</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="81">
       <c r="A11" s="7" t="s">
-        <v>238</v>
+        <v>219</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>237</v>
+        <v>218</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>236</v>
+        <v>217</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>235</v>
+        <v>216</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J11" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="K11" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="K11" s="7" t="s">
-        <v>233</v>
-      </c>
       <c r="L11" s="7" t="s">
-        <v>232</v>
+        <v>213</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>231</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="67.5">
       <c r="A12" s="9" t="s">
-        <v>230</v>
+        <v>211</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>229</v>
+        <v>210</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>228</v>
+        <v>209</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>227</v>
+        <v>208</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>226</v>
+        <v>207</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>225</v>
+        <v>206</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>224</v>
+        <v>205</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>223</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="54">
       <c r="A13" s="7" t="s">
-        <v>222</v>
+        <v>203</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>220</v>
+        <v>201</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>218</v>
+        <v>199</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="40.5">
       <c r="A14" s="7" t="s">
-        <v>252</v>
+        <v>233</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>365</v>
+        <v>346</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>364</v>
+        <v>345</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>363</v>
+        <v>344</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>359</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="40.5">
       <c r="A15" s="9" t="s">
-        <v>259</v>
+        <v>240</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>260</v>
+        <v>241</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>362</v>
+        <v>343</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>361</v>
+        <v>342</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>360</v>
+        <v>341</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>359</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="148.5">
       <c r="A16" s="7" t="s">
-        <v>262</v>
+        <v>243</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>263</v>
+        <v>244</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="F16" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="L16" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J16" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="K16" s="7" t="s">
-        <v>357</v>
-      </c>
-      <c r="L16" s="7" t="s">
-        <v>377</v>
-      </c>
       <c r="M16" s="7" t="s">
-        <v>353</v>
+        <v>334</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="40.5">
       <c r="A17" s="9" t="s">
-        <v>266</v>
+        <v>247</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>267</v>
+        <v>248</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>356</v>
+        <v>337</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>265</v>
+        <v>246</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>355</v>
+        <v>336</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>354</v>
+        <v>335</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>353</v>
+        <v>334</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="40.5">
       <c r="A18" s="7" t="s">
-        <v>268</v>
+        <v>249</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>269</v>
+        <v>250</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>349</v>
+        <v>330</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>352</v>
+        <v>333</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>270</v>
+        <v>251</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>351</v>
+        <v>332</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>350</v>
+        <v>331</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>345</v>
+        <v>326</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="40.5">
       <c r="A19" s="9" t="s">
-        <v>271</v>
+        <v>252</v>
       </c>
       <c r="B19" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>272</v>
-      </c>
       <c r="D19" s="9" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>349</v>
+        <v>330</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>348</v>
+        <v>329</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>270</v>
+        <v>251</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>347</v>
+        <v>328</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>346</v>
+        <v>327</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>345</v>
+        <v>326</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="148.5">
       <c r="A20" s="7" t="s">
-        <v>344</v>
+        <v>325</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>343</v>
+        <v>324</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>312</v>
+        <v>293</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>342</v>
+        <v>323</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>341</v>
+        <v>322</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>340</v>
+        <v>321</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>379</v>
+        <v>360</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>378</v>
+        <v>359</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>380</v>
+        <v>361</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>339</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="81">
       <c r="A21" s="9" t="s">
-        <v>338</v>
+        <v>319</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>337</v>
+        <v>318</v>
       </c>
       <c r="D21" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="I21" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="M21" s="9" t="s">
         <v>312</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>336</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>334</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J21" s="9" t="s">
-        <v>333</v>
-      </c>
-      <c r="K21" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="L21" s="9" t="s">
-        <v>369</v>
-      </c>
-      <c r="M21" s="9" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="54">
       <c r="A22" s="7" t="s">
-        <v>330</v>
+        <v>311</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>329</v>
+        <v>310</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>328</v>
+        <v>309</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>299</v>
+        <v>280</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>327</v>
+        <v>308</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>326</v>
+        <v>307</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>325</v>
+        <v>306</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>370</v>
+        <v>351</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>324</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="54">
       <c r="A23" s="9" t="s">
-        <v>323</v>
+        <v>304</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>322</v>
+        <v>303</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>321</v>
+        <v>302</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>320</v>
+        <v>301</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>319</v>
+        <v>300</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>318</v>
+        <v>299</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>5</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>317</v>
+        <v>298</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>316</v>
+        <v>297</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>371</v>
+        <v>352</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>315</v>
+        <v>296</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="54">
       <c r="A24" s="7" t="s">
-        <v>314</v>
+        <v>295</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="E24" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>311</v>
-      </c>
       <c r="F24" s="7" t="s">
-        <v>310</v>
+        <v>291</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>309</v>
+        <v>290</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>308</v>
+        <v>289</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>307</v>
+        <v>288</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>306</v>
+        <v>287</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>305</v>
+        <v>286</v>
       </c>
       <c r="M24" s="7" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="54">
       <c r="A25" s="9" t="s">
-        <v>303</v>
+        <v>284</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>302</v>
+        <v>283</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>299</v>
+        <v>280</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>298</v>
+        <v>279</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>297</v>
+        <v>278</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>296</v>
+        <v>277</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>295</v>
+        <v>276</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>294</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="54">
       <c r="A26" s="7" t="s">
-        <v>293</v>
+        <v>274</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>290</v>
+        <v>271</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>289</v>
+        <v>270</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>288</v>
+        <v>269</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>287</v>
+        <v>268</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>286</v>
+        <v>267</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>285</v>
+        <v>266</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>283</v>
+        <v>264</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="67.5">
       <c r="A27" s="9" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>279</v>
+        <v>260</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>278</v>
+        <v>259</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>277</v>
+        <v>258</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>276</v>
+        <v>257</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>274</v>
+        <v>255</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>381</v>
+        <v>362</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>273</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update methodology decision table through final evaluation
</commit_message>
<xml_diff>
--- a/methodology/Methodology_Decision_Table.xlsx
+++ b/methodology/Methodology_Decision_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a261b646168a133d/Documents/GitHub/weathering-the-yield/methodology/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="8_{E2880474-6383-4A23-83FB-0BFB047B2884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AA9E37-1F37-4E99-A488-36B950B68385}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="8_{E2880474-6383-4A23-83FB-0BFB047B2884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51683CC6-62D0-4D91-B0F0-54CD06618A2A}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="417">
   <si>
     <t>Senior Thesis Methodology Decision Table</t>
   </si>
@@ -309,9 +309,6 @@
     <t>2022–2025</t>
   </si>
   <si>
-    <t>Proposal; advisor feedback</t>
-  </si>
-  <si>
     <t>Provides four recent future years for final model comparison.</t>
   </si>
   <si>
@@ -411,9 +408,6 @@
     <t>All models must be evaluated on identical observations.</t>
   </si>
   <si>
-    <t>Evaluation script</t>
-  </si>
-  <si>
     <t>M16</t>
   </si>
   <si>
@@ -435,12 +429,6 @@
     <t>County comparisons require enough observed test years to be meaningful.</t>
   </si>
   <si>
-    <t>Evaluation / figures</t>
-  </si>
-  <si>
-    <t>County error maps planned.</t>
-  </si>
-  <si>
     <t>M17</t>
   </si>
   <si>
@@ -450,24 +438,6 @@
     <t>How will geographic model error be examined?</t>
   </si>
   <si>
-    <t>Map county prediction errors and/or changes in county RMSE between model groups</t>
-  </si>
-  <si>
-    <t>He &amp; Luo (2026); Li et al. (2026); Sajid et al. (2022); advisor feedback</t>
-  </si>
-  <si>
-    <t>Identifies locations where models consistently perform poorly or benefit from added weather information.</t>
-  </si>
-  <si>
-    <t>Missing county-year yields must remain visible rather than silently filled.</t>
-  </si>
-  <si>
-    <t>Figures / spatial analysis</t>
-  </si>
-  <si>
-    <t>Exact map statistic can be finalized later.</t>
-  </si>
-  <si>
     <t>M18</t>
   </si>
   <si>
@@ -475,24 +445,6 @@
   </si>
   <si>
     <t>How will meaningful performance differences be assessed?</t>
-  </si>
-  <si>
-    <t>Compare historical vs. conventional-weather models and conventional-weather vs. extreme-weather models using effect size, consistency across years/counties, and an appropriate dependence-aware statistical comparison if feasible</t>
-  </si>
-  <si>
-    <t>Qu et al. (2024); Stracqualursi (2026); advisor feedback</t>
-  </si>
-  <si>
-    <t>RMSE differences alone may not indicate meaningful improvement.</t>
-  </si>
-  <si>
-    <t>County-year errors cannot automatically be treated as independent.</t>
-  </si>
-  <si>
-    <t>Final evaluation script</t>
-  </si>
-  <si>
-    <t>Exact statistical test remains unresolved because the final test period has only four years.</t>
   </si>
   <si>
     <t>M19</t>
@@ -1164,12 +1116,6 @@
     <t>Scripts 17–20 development-stage model evaluation and comparison</t>
   </si>
   <si>
-    <t>Final holdout evaluation workflow following development-stage lock</t>
-  </si>
-  <si>
-    <t>Development-stage algorithm, predictor group, exact model formula, and predictor definitions were formally locked in Script 22 before final holdout evaluation. At the completion of Script 22, the 2022–2025 holdout remained unused.</t>
-  </si>
-  <si>
     <t>Advisor feedback; literature review; Scripts 17–20 development-stage model comparison</t>
   </si>
   <si>
@@ -1179,9 +1125,6 @@
     <t>All nine algorithm × predictor-group specifications were evaluated over the same 2012–2021 validation years. Each pooled specification contained 739 validation observations.</t>
   </si>
   <si>
-    <t>Model selection continued to prioritize pooled RMSE, with MAE used as a complementary error measure and R² treated as secondary. The selected Linear Regression Group 3 specification ranked first among all nine development-stage specifications on pooled RMSE, MAE, and R².</t>
-  </si>
-  <si>
     <t>Multiple Linear Regression, Random Forest, and XGBoost</t>
   </si>
   <si>
@@ -1209,12 +1152,6 @@
     <t>Script 21 was descriptive and diagnostic only and did not trigger predictor, threshold, or model changes. Script 22 formally locked the predictor set and model specification before final holdout evaluation.</t>
   </si>
   <si>
-    <t>Project folders / scripts / methodology decision table / output/development_stage_lock/</t>
-  </si>
-  <si>
-    <t>Script 22 created a machine-readable pre-holdout checkpoint including development_stage_lock.csv, overall_development_ranking.csv, numeric_selection_difference.csv, locked_predictor_definition.csv, development_stage_lock_object.rds, and pre_holdout_checkpoint.csv.</t>
-  </si>
-  <si>
     <t>M23</t>
   </si>
   <si>
@@ -1293,16 +1230,100 @@
     <t>22_development_stage_lock.R; output/development_stage_lock/</t>
   </si>
   <si>
-    <t>Script 22 locked Linear Regression + Group 3. No new model fitting, tuning, or predictor changes occurred in Script 22, and the checkpoint explicitly records final_holdout_used = FALSE.</t>
+    <t>M26</t>
+  </si>
+  <si>
+    <t>Final holdout evaluation</t>
+  </si>
+  <si>
+    <t>How will the locked model be evaluated on the final holdout, and what was the result?</t>
+  </si>
+  <si>
+    <t>Fit the locked Linear Regression Group 3 specification using the complete 2001–2021 development dataset and evaluate it once on the previously untouched 2022–2025 final holdout. Holdout performance will not be used to change the model, predictors, or tuning decisions.</t>
+  </si>
+  <si>
+    <t>Script 22 development-stage lock; Script 23 final holdout evaluation</t>
+  </si>
+  <si>
+    <t>Provides a final out-of-sample assessment of the model selected entirely from pre-2022 development data and evaluates how well the locked specification generalizes to later growing seasons.</t>
+  </si>
+  <si>
+    <t>The 2022–2025 holdout was accessed only after the development-stage specification was formally locked. Holdout results cannot be used for additional tuning, predictor selection, or model-family changes.</t>
+  </si>
+  <si>
+    <t>23_final_holdout_evaluation.R; output/final_holdout_evaluation/</t>
+  </si>
+  <si>
+    <t>The final holdout contained 247 county-year observations across 82 counties. Pooled RMSE = 11.97 bu/acre, MAE = 9.79 bu/acre, and R² = 0.392. Mean residual = 0.794 bu/acre. No model changes were made after holdout evaluation.</t>
+  </si>
+  <si>
+    <t>Proposal; advisor feedback; Scripts 22–23 development-stage lock and final holdout evaluation</t>
+  </si>
+  <si>
+    <t>The 2022–2025 holdout remained unused until the development-stage model was formally locked in Script 22. Script 23 then evaluated the locked Linear Regression Group 3 specification on 247 county-year observations across 82 counties. No post-holdout model or predictor changes were made.</t>
+  </si>
+  <si>
+    <t>Scripts 17–20 development-stage evaluation; Script 23 final holdout evaluation</t>
+  </si>
+  <si>
+    <t>Final holdout evaluation followed the prespecified metric hierarchy. Across 247 holdout observations, RMSE was 11.97 bu/acre, MAE was 9.79 bu/acre, and R² was 0.392. Year-specific metrics were also calculated for 2022–2025.</t>
+  </si>
+  <si>
+    <t>Script 22 locked Linear Regression + Group 3. No new model fitting, tuning, or predictor changes occurred in Script 22, and the checkpoint explicitly records final_holdout_used = FALSE. Script 23 subsequently loaded the saved lock object and used the exact locked formula for final evaluation. The holdout evaluation record confirms model_changed_after_holdout = FALSE.</t>
+  </si>
+  <si>
+    <t>Use county-level error summaries from the 2012–2021 development-stage rolling-validation predictions to examine geographic variation in model performance. Map county RMSE for the selected Linear Regression Group 3 specification and the change in county RMSE from Group 1 to Group 3. Spatial results are descriptive only and will not be used to modify the selected model.</t>
+  </si>
+  <si>
+    <t>He &amp; Luo (2026); Li et al. (2026); Sajid et al. (2022); advisor feedback; Script 17 development-stage validation predictions</t>
+  </si>
+  <si>
+    <t>Development-stage rolling validation provides more repeated evaluation years per county than the four-year final holdout and allows geographic patterns in prediction error and the added value of weather information to be examined more meaningfully.</t>
+  </si>
+  <si>
+    <t>Spatial comparisons use pre-2022 validation predictions only. Spatial results are descriptive and cannot be used for additional feature selection, tuning, or model changes. Counties with fewer observed validation years will be interpreted cautiously rather than treated as having equally precise error estimates.</t>
+  </si>
+  <si>
+    <t>Assess meaningful predictor-group differences using the magnitude and consistency of development-stage predictive performance rather than a formal significance test. Comparisons will use pooled RMSE and MAE differences and percent reductions, year-specific performance differences and win counts, and sensitivity analysis excluding the unusually difficult 2012 validation year.</t>
+  </si>
+  <si>
+    <t>Qu et al. (2024); Stracqualursi (2026); advisor feedback; Scripts 17–20 development-stage model comparisons</t>
+  </si>
+  <si>
+    <t>The research question concerns predictive value rather than statistical significance. Effect magnitude, consistency across rolling-validation years, and sensitivity analyses provide a more appropriate assessment of practical predictive improvement given the limited number of validation years and dependence among county-year errors.</t>
+  </si>
+  <si>
+    <t>All predictor-group comparisons use pre-2022 development-stage validation only. The final 2022–2025 holdout is used only to evaluate the locked model and is not used to reopen predictor-group or model-family comparisons.</t>
+  </si>
+  <si>
+    <t>Scripts 17–20 pooled and yearly performance comparisons, incremental RMSE/MAE comparisons, yearly win counts, and sensitivity analyses</t>
+  </si>
+  <si>
+    <t>No formal p-value-based comparison will be reported. Performance differences will be interpreted in terms of effect magnitude, direction, consistency across years, and robustness to the 2012 sensitivity analysis.</t>
+  </si>
+  <si>
+    <t>24_spatial_error_diagnostic.R; output/spatial_error_diagnostic/</t>
+  </si>
+  <si>
+    <t>Development-stage spatial diagnostic completed using 2012–2021 Linear Regression rolling-validation predictions. Eighty-nine counties had eligible validation observations; Brown, Crawford, and Perry did not. Group 3 produced lower county-level RMSE than Group 1 in 78 of 89 evaluated counties (87.6%). Median county RMSE reduction was 11.33 bu/acre, with a median percentage reduction of 35.7%. Spatial analysis was descriptive only and no model changes were made.</t>
+  </si>
+  <si>
+    <t>Script 23 pooled and year-specific final holdout evaluation; Script 24 county-level development-stage spatial diagnostic</t>
+  </si>
+  <si>
+    <t>Pooled and individual-year performance were evaluated on the 2022–2025 final holdout in Script 23. County-level performance was examined descriptively in Script 24 using 2012–2021 rolling-validation predictions, which provided more repeated observations per county than the four-year holdout. Eighty-nine counties were evaluated, with a median of 9 validation observations per county. The county-level diagnostic was not used to modify the selected model.</t>
+  </si>
+  <si>
+    <t>Project folders / scripts / methodology decision table / output/development_stage_lock/ / output/final_holdout_evaluation/ / output/spatial_error_diagnostic/</t>
+  </si>
+  <si>
+    <t>Script 22 preserved the machine-readable development-stage lock and pre-holdout checkpoint. Script 23 preserved the final fitted model, prediction-level holdout results, pooled and yearly performance metrics, model-fit audit, bias summary, development-versus-holdout comparison, and final diagnostic figures. Script 24 preserved county-level validation coverage, Group 1 versus Group 3 county error comparisons, spatial summary results, and final diagnostic maps.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="mmm\ d\,\ yyyy"/>
-  </numFmts>
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -1426,7 +1447,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1438,9 +1459,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1"/>
@@ -1459,16 +1477,10 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1485,6 +1497,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1550,6 +1574,7 @@
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1603,7 +1628,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MethodologyDecisionsTable" displayName="MethodologyDecisionsTable" ref="A10:K35" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MethodologyDecisionsTable" displayName="MethodologyDecisionsTable" ref="A10:K36" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Decision ID" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Category" dataDxfId="15"/>
@@ -1816,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="11" style="3" customWidth="1"/>
@@ -1834,34 +1859,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14" customHeight="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
     </row>
     <row r="2" spans="1:11" ht="12" customHeight="1">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
     </row>
     <row r="4" spans="1:11" ht="11" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -1870,69 +1895,69 @@
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
     </row>
     <row r="5" spans="1:11" ht="14" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(E11:E35,"Final")</f>
-        <v>24</v>
-      </c>
-      <c r="D5" s="19" t="s">
+        <f>COUNTIF(E11:E36,"Final")</f>
+        <v>26</v>
+      </c>
+      <c r="D5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
     </row>
     <row r="6" spans="1:11" ht="14" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF(E11:E35,"Provisional")</f>
-        <v>1</v>
-      </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
+        <f>COUNTIF(E11:E36,"Provisional")</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
     </row>
     <row r="7" spans="1:11" ht="14" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(E11:E35,"Needs Advisor Input")</f>
+        <f>COUNTIF(E11:E36,"Needs Advisor Input")</f>
         <v>0</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
     </row>
     <row r="10" spans="1:11" ht="18" customHeight="1">
       <c r="A10" s="2" t="s">
@@ -1997,7 +2022,7 @@
       <c r="I11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="12">
         <v>46279</v>
       </c>
       <c r="K11" s="4" t="s">
@@ -2032,7 +2057,7 @@
       <c r="I12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="12">
         <v>46279</v>
       </c>
       <c r="K12" s="4" t="s">
@@ -2067,7 +2092,7 @@
       <c r="I13" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="12">
         <v>46279</v>
       </c>
       <c r="K13" s="4" t="s">
@@ -2102,7 +2127,7 @@
       <c r="I14" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="12">
         <v>46279</v>
       </c>
       <c r="K14" s="4" t="s">
@@ -2117,10 +2142,10 @@
         <v>57</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>5</v>
@@ -2129,19 +2154,19 @@
         <v>58</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="J15" s="5">
+        <v>167</v>
+      </c>
+      <c r="J15" s="12">
         <v>46266</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>347</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="175.5">
@@ -2152,31 +2177,31 @@
         <v>60</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="J16" s="5">
+        <v>174</v>
+      </c>
+      <c r="J16" s="12">
         <v>46266</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="40.5">
@@ -2207,7 +2232,7 @@
       <c r="I17" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="J17" s="5"/>
+      <c r="J17" s="12"/>
       <c r="K17" s="4" t="s">
         <v>69</v>
       </c>
@@ -2223,28 +2248,28 @@
         <v>72</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>353</v>
+        <v>337</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>355</v>
+        <v>339</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>354</v>
+        <v>338</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>73</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="J18" s="5">
+        <v>341</v>
+      </c>
+      <c r="J18" s="12">
         <v>46287</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>356</v>
+        <v>340</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="40.5">
@@ -2275,7 +2300,7 @@
       <c r="I19" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="J19" s="5"/>
+      <c r="J19" s="12"/>
       <c r="K19" s="4" t="s">
         <v>82</v>
       </c>
@@ -2291,7 +2316,7 @@
         <v>85</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>363</v>
+        <v>347</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>5</v>
@@ -2300,22 +2325,22 @@
         <v>86</v>
       </c>
       <c r="G20" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I20" s="4" t="s">
         <v>348</v>
       </c>
-      <c r="H20" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="J20" s="5">
+      <c r="J20" s="12">
         <v>46279</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="94.5">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="108">
       <c r="A21" s="4" t="s">
         <v>87</v>
       </c>
@@ -2332,526 +2357,563 @@
         <v>5</v>
       </c>
       <c r="F21" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="H21" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="4" t="s">
-        <v>93</v>
-      </c>
       <c r="I21" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="J21" s="5">
+        <v>391</v>
+      </c>
+      <c r="J21" s="12">
         <v>46279</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>366</v>
+        <v>397</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="40.5">
       <c r="A22" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F22" s="4" t="s">
+      <c r="G22" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="H22" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="I22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="J22" s="12">
+        <v>46279</v>
+      </c>
+      <c r="K22" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="J22" s="5">
-        <v>46279</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="67.5">
       <c r="A23" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="C23" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>367</v>
-      </c>
-      <c r="G23" s="4" t="s">
+      <c r="H23" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="H23" s="4" t="s">
-        <v>108</v>
-      </c>
       <c r="I23" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="J23" s="5">
+        <v>350</v>
+      </c>
+      <c r="J23" s="12">
         <v>46279</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="40.5">
       <c r="A24" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="C24" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="E24" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F24" s="4" t="s">
+      <c r="G24" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="H24" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="I24" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="J24" s="12">
+        <v>46279</v>
+      </c>
+      <c r="K24" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="J24" s="5">
+    </row>
+    <row r="25" spans="1:11" ht="81">
+      <c r="A25" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="J25" s="12">
         <v>46279</v>
       </c>
-      <c r="K24" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="108">
-      <c r="A25" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="H25" s="4" t="s">
+      <c r="K25" s="4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="162">
+      <c r="A26" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="B26" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="J25" s="5">
+      <c r="C26" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="J26" s="12">
         <v>46279</v>
       </c>
-      <c r="K25" s="4" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="40.5">
-      <c r="A26" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="G26" s="4" t="s">
+      <c r="K26" s="4" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="175.5">
+      <c r="A27" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="B27" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="C27" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="J26" s="5">
-        <v>46279</v>
-      </c>
-      <c r="K26" s="4" t="s">
+      <c r="D27" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="J27" s="12">
+        <v>46313</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="121.5">
+      <c r="A28" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" ht="40.5">
-      <c r="A27" s="4" t="s">
+      <c r="B28" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="C28" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="I27" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="J27" s="5">
-        <v>46279</v>
-      </c>
-      <c r="K27" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="81">
-      <c r="A28" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>146</v>
-      </c>
       <c r="D28" s="4" t="s">
-        <v>147</v>
+        <v>405</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>148</v>
+        <v>406</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>149</v>
+        <v>407</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>150</v>
+        <v>408</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="J28" s="5"/>
+        <v>409</v>
+      </c>
+      <c r="J28" s="12">
+        <v>46313</v>
+      </c>
       <c r="K28" s="4" t="s">
-        <v>152</v>
+        <v>410</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="67.5">
       <c r="A29" s="4" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>371</v>
+        <v>352</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>372</v>
+        <v>353</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>373</v>
+        <v>354</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>374</v>
+        <v>355</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>375</v>
-      </c>
-      <c r="J29" s="5">
+        <v>356</v>
+      </c>
+      <c r="J29" s="12">
         <v>46302</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>376</v>
+        <v>357</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="81">
       <c r="A30" s="4" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>377</v>
+        <v>358</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="J30" s="5">
+        <v>359</v>
+      </c>
+      <c r="J30" s="12">
         <v>46279</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>379</v>
+        <v>360</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="40.5">
       <c r="A31" s="4" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>166</v>
+        <v>150</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="J31" s="5">
+        <v>153</v>
+      </c>
+      <c r="J31" s="12">
         <v>46279</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="108">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="175.5">
       <c r="A32" s="4" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>380</v>
-      </c>
-      <c r="J32" s="5">
+        <v>415</v>
+      </c>
+      <c r="J32" s="12">
         <v>46279</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>381</v>
+        <v>416</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="148.5">
       <c r="A33" s="4" t="s">
-        <v>382</v>
+        <v>361</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>383</v>
+        <v>362</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>384</v>
+        <v>363</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>385</v>
+        <v>364</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>386</v>
+        <v>365</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>387</v>
+        <v>366</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>388</v>
+        <v>367</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>389</v>
-      </c>
-      <c r="J33" s="5">
+        <v>368</v>
+      </c>
+      <c r="J33" s="12">
         <v>46302</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>390</v>
+        <v>369</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="94.5">
       <c r="A34" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="J34" s="12">
+        <v>46302</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="135">
+      <c r="A35" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="J35" s="12">
+        <v>46302</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="94.5">
+      <c r="A36" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="G36" s="3" t="s">
         <v>392</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="H36" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="I36" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="E34" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F34" s="4" t="s">
+      <c r="J36" s="11">
+        <v>46313</v>
+      </c>
+      <c r="K36" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="G34" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="H34" s="4" t="s">
-        <v>397</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="J34" s="5">
-        <v>46302</v>
-      </c>
-      <c r="K34" s="4" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="81">
-      <c r="A35" s="4" t="s">
-        <v>400</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>402</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>405</v>
-      </c>
-      <c r="H35" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>407</v>
-      </c>
-      <c r="J35" s="5">
-        <v>46302</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="18" customHeight="1">
-      <c r="A37" s="20" t="s">
-        <v>178</v>
-      </c>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="20"/>
-      <c r="H37" s="20"/>
-      <c r="I37" s="20"/>
-      <c r="J37" s="20"/>
-      <c r="K37" s="20"/>
+    </row>
+    <row r="38" spans="1:11" ht="18" customHeight="1">
+      <c r="A38" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2859,9 +2921,9 @@
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="D4:K4"/>
     <mergeCell ref="D5:K7"/>
-    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A38:K38"/>
   </mergeCells>
-  <conditionalFormatting sqref="E11:E35">
+  <conditionalFormatting sqref="E11:E36">
     <cfRule type="expression" dxfId="5" priority="1">
       <formula>E11="Final"</formula>
     </cfRule>
@@ -2873,7 +2935,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="E11:E35" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="E11:E36" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Final,Provisional,Needs Advisor Input"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2890,869 +2952,869 @@
   <dimension ref="A1:M27"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="11" style="6" customWidth="1"/>
-    <col min="2" max="2" width="18" style="6" customWidth="1"/>
-    <col min="3" max="4" width="28" style="6" customWidth="1"/>
-    <col min="5" max="5" width="20" style="6" customWidth="1"/>
-    <col min="6" max="6" width="38" style="6" customWidth="1"/>
-    <col min="7" max="7" width="16" style="6" customWidth="1"/>
-    <col min="8" max="8" width="34" style="6" customWidth="1"/>
-    <col min="9" max="9" width="14" style="6" customWidth="1"/>
-    <col min="10" max="10" width="30" style="6" customWidth="1"/>
-    <col min="11" max="11" width="38" style="6" customWidth="1"/>
-    <col min="12" max="13" width="40" style="6" customWidth="1"/>
-    <col min="14" max="16384" width="9" style="6"/>
+    <col min="1" max="1" width="11" style="5" customWidth="1"/>
+    <col min="2" max="2" width="18" style="5" customWidth="1"/>
+    <col min="3" max="4" width="28" style="5" customWidth="1"/>
+    <col min="5" max="5" width="20" style="5" customWidth="1"/>
+    <col min="6" max="6" width="38" style="5" customWidth="1"/>
+    <col min="7" max="7" width="16" style="5" customWidth="1"/>
+    <col min="8" max="8" width="34" style="5" customWidth="1"/>
+    <col min="9" max="9" width="14" style="5" customWidth="1"/>
+    <col min="10" max="10" width="30" style="5" customWidth="1"/>
+    <col min="11" max="11" width="38" style="5" customWidth="1"/>
+    <col min="12" max="13" width="40" style="5" customWidth="1"/>
+    <col min="14" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="14" customHeight="1">
-      <c r="A1" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
+      <c r="A1" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
     </row>
     <row r="2" spans="1:13" ht="11" customHeight="1">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
     </row>
     <row r="4" spans="1:13" ht="27.75">
-      <c r="A4" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
     </row>
     <row r="5" spans="1:13" ht="14" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="6">
+      <c r="A5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5">
         <f>COUNTIF(I11:I200,"Final")</f>
         <v>12</v>
       </c>
-      <c r="D5" s="15" t="s">
-        <v>230</v>
-      </c>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
+      <c r="D5" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
     </row>
     <row r="6" spans="1:13" ht="14" customHeight="1">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <f>COUNTIF(I11:I200,"Provisional")</f>
         <v>0</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
     </row>
     <row r="7" spans="1:13" ht="14" customHeight="1">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" s="5">
+        <f>COUNTIF(I11:I200,"Excluded")</f>
+        <v>5</v>
+      </c>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+    </row>
+    <row r="10" spans="1:13" ht="16.05" customHeight="1">
+      <c r="A10" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="81">
+      <c r="A11" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="67.5">
+      <c r="A12" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="M12" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="54">
+      <c r="A13" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="40.5">
+      <c r="A14" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="40.5">
+      <c r="A15" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="L15" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="148.5">
+      <c r="A16" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="B7" s="6">
-        <f>COUNTIF(I11:I200,"Excluded")</f>
-        <v>5</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="15"/>
-      <c r="M7" s="15"/>
-    </row>
-    <row r="10" spans="1:13" ht="16.05" customHeight="1">
-      <c r="A10" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="C10" s="10" t="s">
+      <c r="F16" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="40.5">
+      <c r="A17" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="G10" s="10" t="s">
+      <c r="E17" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J17" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="H10" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="I10" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="J10" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="K10" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="M10" s="10" t="s">
+      <c r="K17" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="M17" s="8" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="40.5">
+      <c r="A18" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" ht="81">
-      <c r="A11" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="C11" s="7" t="s">
+      <c r="E18" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="40.5">
+      <c r="A19" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="L11" s="7" t="s">
+      <c r="C19" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="148.5">
+      <c r="A20" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="I20" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="M11" s="7" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="67.5">
-      <c r="A12" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="M12" s="9" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="54">
-      <c r="A13" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="M13" s="7" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="40.5">
-      <c r="A14" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="F14" s="7" t="s">
+      <c r="J20" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="81">
+      <c r="A21" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="L21" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="M21" s="8" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="54">
+      <c r="A22" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="M22" s="6" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="54">
+      <c r="A23" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="L23" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="M23" s="8" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="54">
+      <c r="A24" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="M24" s="6" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="54">
+      <c r="A25" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="54">
+      <c r="A26" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="M26" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="67.5">
+      <c r="A27" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="L27" s="8" t="s">
         <v>346</v>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="H14" s="7" t="s">
+      <c r="M27" s="8" t="s">
         <v>238</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L14" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="M14" s="7" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="40.5">
-      <c r="A15" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>343</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J15" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="K15" s="9" t="s">
-        <v>342</v>
-      </c>
-      <c r="L15" s="9" t="s">
-        <v>341</v>
-      </c>
-      <c r="M15" s="9" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="148.5">
-      <c r="A16" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J16" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="K16" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="L16" s="7" t="s">
-        <v>358</v>
-      </c>
-      <c r="M16" s="7" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="40.5">
-      <c r="A17" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>337</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J17" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="K17" s="9" t="s">
-        <v>336</v>
-      </c>
-      <c r="L17" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="M17" s="9" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="40.5">
-      <c r="A18" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="I18" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="40.5">
-      <c r="A19" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>330</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="I19" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J19" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="K19" s="9" t="s">
-        <v>328</v>
-      </c>
-      <c r="L19" s="9" t="s">
-        <v>327</v>
-      </c>
-      <c r="M19" s="9" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="148.5">
-      <c r="A20" s="7" t="s">
-        <v>325</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>360</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>359</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>361</v>
-      </c>
-      <c r="M20" s="7" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="81">
-      <c r="A21" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>318</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>317</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>316</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J21" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="K21" s="9" t="s">
-        <v>313</v>
-      </c>
-      <c r="L21" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="M21" s="9" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="54">
-      <c r="A22" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>282</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>280</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>308</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="K22" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="L22" s="7" t="s">
-        <v>351</v>
-      </c>
-      <c r="M22" s="7" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="54">
-      <c r="A23" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>303</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>302</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>301</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>300</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>299</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J23" s="9" t="s">
-        <v>298</v>
-      </c>
-      <c r="K23" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="L23" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="M23" s="9" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="54">
-      <c r="A24" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>289</v>
-      </c>
-      <c r="I24" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>288</v>
-      </c>
-      <c r="K24" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="L24" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="M24" s="7" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="54">
-      <c r="A25" s="9" t="s">
-        <v>284</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>280</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>279</v>
-      </c>
-      <c r="I25" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="J25" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="K25" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="L25" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="M25" s="9" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="54">
-      <c r="A26" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="I26" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="L26" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="M26" s="7" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" ht="67.5">
-      <c r="A27" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>258</v>
-      </c>
-      <c r="G27" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="I27" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="J27" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="K27" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="L27" s="9" t="s">
-        <v>362</v>
-      </c>
-      <c r="M27" s="9" t="s">
-        <v>254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>